<commit_message>
ordering fixes and delta method implemented for all methods
</commit_message>
<xml_diff>
--- a/examples/output/LC2_routeChoice.xlsx
+++ b/examples/output/LC2_routeChoice.xlsx
@@ -507,25 +507,25 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>-0.044835691282718415</v>
+        <v>-0.04483569128271805</v>
       </c>
       <c r="C2">
-        <v>0.048013111629023296</v>
+        <v>0.0480131116290233</v>
       </c>
       <c r="D2">
-        <v>-0.9338218199466961</v>
+        <v>-0.9338218199466883</v>
       </c>
       <c r="E2">
-        <v>0.35039581205625914</v>
+        <v>0.3503958120562629</v>
       </c>
       <c r="F2">
-        <v>0.052664896401448294</v>
+        <v>0.052664896401448315</v>
       </c>
       <c r="G2">
-        <v>-0.8513392097261474</v>
+        <v>-0.8513392097261401</v>
       </c>
       <c r="H2">
-        <v>0.39458094995746285</v>
+        <v>0.39458094995746684</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -559,22 +559,22 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>-2.167558634956704</v>
+        <v>-2.1675586349567024</v>
       </c>
       <c r="C4">
-        <v>0.18482510938414767</v>
+        <v>0.184825109384147</v>
       </c>
       <c r="D4">
-        <v>-11.727619922310264</v>
+        <v>-11.727619922310298</v>
       </c>
       <c r="E4">
         <v>0.0</v>
       </c>
       <c r="F4">
-        <v>0.28956752030507027</v>
+        <v>0.289567520305068</v>
       </c>
       <c r="G4">
-        <v>-7.485503321205015</v>
+        <v>-7.485503321205068</v>
       </c>
       <c r="H4">
         <v>7.127631818093505e-14</v>
@@ -585,25 +585,25 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>-0.7637913866594699</v>
+        <v>-0.7637913866594704</v>
       </c>
       <c r="C5">
-        <v>0.1048832100037416</v>
+        <v>0.10488321000374203</v>
       </c>
       <c r="D5">
-        <v>-7.2823036845670766</v>
+        <v>-7.282303684567052</v>
       </c>
       <c r="E5">
         <v>3.2818192607919627e-13</v>
       </c>
       <c r="F5">
-        <v>0.28232382087178187</v>
+        <v>0.28232382087178515</v>
       </c>
       <c r="G5">
-        <v>-2.7053735115264956</v>
+        <v>-2.7053735115264663</v>
       </c>
       <c r="H5">
-        <v>0.006822762629299373</v>
+        <v>0.006822762629300039</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -614,19 +614,19 @@
         <v>-0.04748197061302284</v>
       </c>
       <c r="C6">
-        <v>0.005676104686183819</v>
+        <v>0.005676104686183827</v>
       </c>
       <c r="D6">
-        <v>-8.365238704740328</v>
+        <v>-8.365238704740317</v>
       </c>
       <c r="E6">
         <v>0.0</v>
       </c>
       <c r="F6">
-        <v>0.010465380650801976</v>
+        <v>0.010465380650802042</v>
       </c>
       <c r="G6">
-        <v>-4.537051464954047</v>
+        <v>-4.5370514649540175</v>
       </c>
       <c r="H6">
         <v>5.704618906809955e-6</v>
@@ -637,22 +637,22 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>-0.039622321680761075</v>
+        <v>-0.03962232168076108</v>
       </c>
       <c r="C7">
-        <v>0.003892685285585306</v>
+        <v>0.0038926852855853144</v>
       </c>
       <c r="D7">
-        <v>-10.178660429468405</v>
+        <v>-10.178660429468385</v>
       </c>
       <c r="E7">
         <v>0.0</v>
       </c>
       <c r="F7">
-        <v>0.007927293689730802</v>
+        <v>0.007927293689730866</v>
       </c>
       <c r="G7">
-        <v>-4.998215435374715</v>
+        <v>-4.998215435374676</v>
       </c>
       <c r="H7">
         <v>5.786331791490795e-7</v>
@@ -663,25 +663,25 @@
         <v>14</v>
       </c>
       <c r="B8">
-        <v>-0.5334238154537838</v>
+        <v>-0.5334238154537845</v>
       </c>
       <c r="C8">
-        <v>0.0935585247593437</v>
+        <v>0.09355852475934409</v>
       </c>
       <c r="D8">
-        <v>-5.70149878726589</v>
+        <v>-5.701498787265873</v>
       </c>
       <c r="E8">
         <v>1.1875858074716916e-8</v>
       </c>
       <c r="F8">
-        <v>0.25572873231201393</v>
+        <v>0.25572873231201676</v>
       </c>
       <c r="G8">
-        <v>-2.0858970778573087</v>
+        <v>-2.0858970778572883</v>
       </c>
       <c r="H8">
-        <v>0.0369879470533645</v>
+        <v>0.03698794705336628</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -689,22 +689,22 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-0.09571692658722442</v>
+        <v>-0.0957169265872244</v>
       </c>
       <c r="C9">
-        <v>0.01625135525388701</v>
+        <v>0.01625135525388702</v>
       </c>
       <c r="D9">
-        <v>-5.889781196207053</v>
+        <v>-5.889781196207048</v>
       </c>
       <c r="E9">
         <v>3.867072884133904e-9</v>
       </c>
       <c r="F9">
-        <v>0.024211051083158516</v>
+        <v>0.024211051083158595</v>
       </c>
       <c r="G9">
-        <v>-3.9534395371131246</v>
+        <v>-3.953439537113111</v>
       </c>
       <c r="H9">
         <v>7.703573699613386e-5</v>
@@ -715,22 +715,22 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>-0.09772593406430348</v>
+        <v>-0.09772593406430363</v>
       </c>
       <c r="C10">
-        <v>0.014144364741426227</v>
+        <v>0.014144364741426248</v>
       </c>
       <c r="D10">
-        <v>-6.909178026078633</v>
+        <v>-6.909178026078634</v>
       </c>
       <c r="E10">
         <v>4.874767256524137e-12</v>
       </c>
       <c r="F10">
-        <v>0.030424983142569924</v>
+        <v>0.03042498314257006</v>
       </c>
       <c r="G10">
-        <v>-3.212029193454758</v>
+        <v>-3.212029193454749</v>
       </c>
       <c r="H10">
         <v>0.0013180098134544238</v>
@@ -741,22 +741,22 @@
         <v>17</v>
       </c>
       <c r="B11">
-        <v>-0.0735490626403853</v>
+        <v>-0.07354906264038533</v>
       </c>
       <c r="C11">
-        <v>0.00855815924675458</v>
+        <v>0.008558159246754581</v>
       </c>
       <c r="D11">
-        <v>-8.59402828572938</v>
+        <v>-8.594028285729381</v>
       </c>
       <c r="E11">
         <v>0.0</v>
       </c>
       <c r="F11">
-        <v>0.017977995268665666</v>
+        <v>0.017977995268665718</v>
       </c>
       <c r="G11">
-        <v>-4.091060295725851</v>
+        <v>-4.09106029572584</v>
       </c>
       <c r="H11">
         <v>4.2940546177261396e-5</v>
@@ -767,25 +767,25 @@
         <v>18</v>
       </c>
       <c r="B12">
-        <v>-0.03917735724257422</v>
+        <v>-0.03917735724257428</v>
       </c>
       <c r="C12">
-        <v>0.2675779176725525</v>
+        <v>0.2675779176725529</v>
       </c>
       <c r="D12">
-        <v>-0.14641476241143847</v>
+        <v>-0.1464147624114385</v>
       </c>
       <c r="E12">
-        <v>0.8835939741752001</v>
+        <v>0.8835939741751999</v>
       </c>
       <c r="F12">
-        <v>0.683303955316365</v>
+        <v>0.6833039553163706</v>
       </c>
       <c r="G12">
-        <v>-0.05733518288275585</v>
+        <v>-0.05733518288275548</v>
       </c>
       <c r="H12">
-        <v>0.9542781945502756</v>
+        <v>0.9542781945502758</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -829,7 +829,7 @@
         <v>20</v>
       </c>
       <c r="B1">
-        <v>-1564.0986680403835</v>
+        <v>-1564.0986680403832</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -869,7 +869,7 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>1.279310941696167</v>
+        <v>1.2846930027008057</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -893,7 +893,7 @@
         <v>29</v>
       </c>
       <c r="B9">
-        <v>3148.197336080767</v>
+        <v>3148.1973360807665</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -901,7 +901,7 @@
         <v>30</v>
       </c>
       <c r="B10">
-        <v>3209.779635250362</v>
+        <v>3209.7796352503615</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -909,7 +909,7 @@
         <v>31</v>
       </c>
       <c r="B11">
-        <v>0.3538037251308934</v>
+        <v>0.35380372513089353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>